<commit_message>
Automate leak-event inversion workflow - Add scripts for abnormal high concentration detection and batch leak inversion - Move runnable data extraction workflows into scripts/ - Support pollutant metadata in concentration outputs for result naming - Copy training input Excel files into each result directory - Save and auto-close visualization outputs during batch runs - Add timestamp/pollutant-based result folders and per-run logs
</commit_message>
<xml_diff>
--- a/data/shsh_js/wind.xlsx
+++ b/data/shsh_js/wind.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C26"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -439,277 +439,145 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46068.66666666666</v>
+        <v>46126.33333333334</v>
       </c>
       <c r="B2" t="n">
-        <v>91</v>
+        <v>309</v>
       </c>
       <c r="C2" t="n">
-        <v>2.7</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>46068.70833333334</v>
+        <v>46126.375</v>
       </c>
       <c r="B3" t="n">
-        <v>90</v>
+        <v>292</v>
       </c>
       <c r="C3" t="n">
-        <v>2.5</v>
+        <v>2.9</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>46068.75</v>
+        <v>46126.41666666666</v>
       </c>
       <c r="B4" t="n">
-        <v>81</v>
+        <v>294</v>
       </c>
       <c r="C4" t="n">
-        <v>2.4</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>46068.79166666666</v>
+        <v>46126.45833333334</v>
       </c>
       <c r="B5" t="n">
-        <v>75</v>
+        <v>294</v>
       </c>
       <c r="C5" t="n">
-        <v>2.6</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>46068.83333333334</v>
+        <v>46126.5</v>
       </c>
       <c r="B6" t="n">
-        <v>64</v>
+        <v>294</v>
       </c>
       <c r="C6" t="n">
-        <v>2.8</v>
+        <v>3.8</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>46068.875</v>
+        <v>46126.54166666666</v>
       </c>
       <c r="B7" t="n">
-        <v>58.99999999999999</v>
+        <v>298.9999999999999</v>
       </c>
       <c r="C7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>46068.91666666666</v>
+        <v>46126.58333333334</v>
       </c>
       <c r="B8" t="n">
-        <v>50.99999999999999</v>
+        <v>312.9999999999999</v>
       </c>
       <c r="C8" t="n">
-        <v>3.8</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>46068.95833333334</v>
+        <v>46126.625</v>
       </c>
       <c r="B9" t="n">
-        <v>40</v>
+        <v>309</v>
       </c>
       <c r="C9" t="n">
-        <v>3.8</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>46069</v>
+        <v>46126.66666666666</v>
       </c>
       <c r="B10" t="n">
-        <v>45</v>
+        <v>297</v>
       </c>
       <c r="C10" t="n">
-        <v>3.2</v>
+        <v>3.9</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>46069.04166666666</v>
+        <v>46126.70833333334</v>
       </c>
       <c r="B11" t="n">
-        <v>40.99999999999999</v>
+        <v>297</v>
       </c>
       <c r="C11" t="n">
-        <v>3.9</v>
+        <v>3.8</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>46069.08333333334</v>
+        <v>46126.75</v>
       </c>
       <c r="B12" t="n">
-        <v>42</v>
+        <v>289</v>
       </c>
       <c r="C12" t="n">
-        <v>3.4</v>
+        <v>3.1</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>46069.125</v>
+        <v>46126.79166666666</v>
       </c>
       <c r="B13" t="n">
-        <v>26</v>
+        <v>277</v>
       </c>
       <c r="C13" t="n">
-        <v>3.8</v>
+        <v>2.9</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>46069.16666666666</v>
+        <v>46126.83333333334</v>
       </c>
       <c r="B14" t="n">
-        <v>17</v>
+        <v>279</v>
       </c>
       <c r="C14" t="n">
-        <v>3.3</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="1" t="n">
-        <v>46069.20833333334</v>
-      </c>
-      <c r="B15" t="n">
-        <v>27</v>
-      </c>
-      <c r="C15" t="n">
-        <v>4.3</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="1" t="n">
-        <v>46069.25</v>
-      </c>
-      <c r="B16" t="n">
-        <v>15</v>
-      </c>
-      <c r="C16" t="n">
-        <v>3.1</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="1" t="n">
-        <v>46069.29166666666</v>
-      </c>
-      <c r="B17" t="n">
-        <v>25</v>
-      </c>
-      <c r="C17" t="n">
-        <v>2.4</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="1" t="n">
-        <v>46069.33333333334</v>
-      </c>
-      <c r="B18" t="n">
-        <v>25</v>
-      </c>
-      <c r="C18" t="n">
-        <v>3.5</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="1" t="n">
-        <v>46069.375</v>
-      </c>
-      <c r="B19" t="n">
-        <v>16</v>
-      </c>
-      <c r="C19" t="n">
-        <v>3.3</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="1" t="n">
-        <v>46069.41666666666</v>
-      </c>
-      <c r="B20" t="n">
-        <v>13</v>
-      </c>
-      <c r="C20" t="n">
-        <v>2.2</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="1" t="n">
-        <v>46069.45833333334</v>
-      </c>
-      <c r="B21" t="n">
-        <v>2</v>
-      </c>
-      <c r="C21" t="n">
         <v>2.5</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="1" t="n">
-        <v>46069.5</v>
-      </c>
-      <c r="B22" t="n">
-        <v>6</v>
-      </c>
-      <c r="C22" t="n">
-        <v>2.7</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="1" t="n">
-        <v>46069.54166666666</v>
-      </c>
-      <c r="B23" t="n">
-        <v>4</v>
-      </c>
-      <c r="C23" t="n">
-        <v>2.1</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="1" t="n">
-        <v>46069.58333333334</v>
-      </c>
-      <c r="B24" t="n">
-        <v>7</v>
-      </c>
-      <c r="C24" t="n">
-        <v>1.7</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="1" t="n">
-        <v>46069.625</v>
-      </c>
-      <c r="B25" t="n">
-        <v>340</v>
-      </c>
-      <c r="C25" t="n">
-        <v>2.2</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="1" t="n">
-        <v>46069.66666666666</v>
-      </c>
-      <c r="B26" t="n">
-        <v>345</v>
-      </c>
-      <c r="C26" t="n">
-        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>